<commit_message>
added select all product wishlist
</commit_message>
<xml_diff>
--- a/public/downloads/product_upload.xlsx
+++ b/public/downloads/product_upload.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ekmatra\public\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{750EB514-AF3A-406D-955F-03A81A2ECE18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{70E1FF9E-4614-4AEC-BB1E-42BC343E4F58}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10305"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Name</t>
   </si>
@@ -82,18 +81,12 @@
   </si>
   <si>
     <t>http://ekmatra.in/product/168191451417316.png</t>
-  </si>
-  <si>
-    <t>specification</t>
-  </si>
-  <si>
-    <t>Dial Type:Square,Screen Type:IPS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -457,14 +450,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D18B06-EA8D-4AB8-B87F-67F942C2DE80}">
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="47.26953125" customWidth="1"/>
+    <col min="5" max="5" width="47.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
@@ -495,11 +488,8 @@
       <c r="J1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K1" t="s">
-        <v>16</v>
-      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -529,14 +519,11 @@
       </c>
       <c r="J2" t="s">
         <v>5</v>
-      </c>
-      <c r="K2" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{4F8CFEEC-ECC4-4874-8AFD-0A1FC98ECCCC}"/>
+    <hyperlink ref="E2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>